<commit_message>
Update the data dicotnary to have scales
</commit_message>
<xml_diff>
--- a/data/data-templates/GLATAR_full_data_dictionary.xlsx
+++ b/data/data-templates/GLATAR_full_data_dictionary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/data/data-templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777C8AE5-D60F-E44D-86F7-002C6F436596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF067D3-25A3-7F4E-B27A-92A767F00A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19500" xr2:uid="{40342B9E-7668-1F40-BC40-905B8062AAFC}"/>
   </bookViews>
@@ -443,9 +443,6 @@
     <t>Type of tissue collected (e.g., muscle, fin clip)</t>
   </si>
   <si>
-    <t>belly flap, blood, carcass, cleithra, eye lens, egg, fin, gonad, heart, liver, muscle, otolith, scale, spine, stomach, viscera, whole body, whole body (gonads removed), or whole body (stomach removed)</t>
-  </si>
-  <si>
     <t xml:space="preserve">sample_procedure </t>
   </si>
   <si>
@@ -1170,6 +1167,9 @@
   </si>
   <si>
     <t xml:space="preserve">egg, fry, larva, nymph, pupa, juvenile, or adult </t>
+  </si>
+  <si>
+    <t>belly flap, blood, carcass, cleithra, eye lens, egg, fin, gonad, heart, liver, muscle, otolith, scales, spine, stomach, viscera, whole body, whole body (gonads removed), or whole body (stomach removed)</t>
   </si>
 </sst>
 </file>
@@ -2201,7 +2201,7 @@
       </c>
       <c r="E29" s="9"/>
       <c r="F29" s="15" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="140" x14ac:dyDescent="0.2">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="E30" s="9"/>
       <c r="F30" s="15" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
@@ -2243,13 +2243,13 @@
         <v>66</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C32" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>305</v>
-      </c>
-      <c r="D32" s="9" t="s">
-        <v>306</v>
       </c>
       <c r="E32" s="9"/>
       <c r="F32" s="9"/>
@@ -2259,13 +2259,13 @@
         <v>66</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C33" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="D33" s="9" t="s">
         <v>307</v>
-      </c>
-      <c r="D33" s="9" t="s">
-        <v>308</v>
       </c>
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
@@ -2291,13 +2291,13 @@
         <v>66</v>
       </c>
       <c r="B35" s="9" t="s">
+        <v>308</v>
+      </c>
+      <c r="C35" s="9" t="s">
         <v>309</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="D35" s="9" t="s">
         <v>310</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>311</v>
       </c>
       <c r="E35" s="9"/>
       <c r="F35" s="9"/>
@@ -2307,13 +2307,13 @@
         <v>66</v>
       </c>
       <c r="B36" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="C36" s="9" t="s">
         <v>312</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="D36" s="9" t="s">
         <v>313</v>
-      </c>
-      <c r="D36" s="9" t="s">
-        <v>314</v>
       </c>
       <c r="E36" s="9"/>
       <c r="F36" s="9"/>
@@ -2323,13 +2323,13 @@
         <v>66</v>
       </c>
       <c r="B37" s="25" t="s">
+        <v>314</v>
+      </c>
+      <c r="C37" s="9" t="s">
         <v>315</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="D37" s="9" t="s">
         <v>316</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>317</v>
       </c>
       <c r="E37" s="9"/>
       <c r="F37" s="9"/>
@@ -2339,13 +2339,13 @@
         <v>66</v>
       </c>
       <c r="B38" s="25" t="s">
+        <v>317</v>
+      </c>
+      <c r="C38" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="D38" s="9" t="s">
         <v>319</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>320</v>
       </c>
       <c r="E38" s="9"/>
       <c r="F38" s="9"/>
@@ -2355,13 +2355,13 @@
         <v>66</v>
       </c>
       <c r="B39" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="C39" s="9" t="s">
         <v>321</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="D39" s="9" t="s">
         <v>322</v>
-      </c>
-      <c r="D39" s="9" t="s">
-        <v>323</v>
       </c>
       <c r="E39" s="9"/>
       <c r="F39" s="9"/>
@@ -2371,13 +2371,13 @@
         <v>66</v>
       </c>
       <c r="B40" s="25" t="s">
+        <v>323</v>
+      </c>
+      <c r="C40" s="9" t="s">
         <v>324</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="D40" s="9" t="s">
         <v>325</v>
-      </c>
-      <c r="D40" s="9" t="s">
-        <v>326</v>
       </c>
       <c r="E40" s="9"/>
       <c r="F40" s="9"/>
@@ -2387,13 +2387,13 @@
         <v>66</v>
       </c>
       <c r="B41" s="25" t="s">
+        <v>326</v>
+      </c>
+      <c r="C41" s="9" t="s">
         <v>327</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="D41" s="9" t="s">
         <v>328</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>329</v>
       </c>
       <c r="E41" s="9"/>
       <c r="F41" s="9"/>
@@ -2403,13 +2403,13 @@
         <v>66</v>
       </c>
       <c r="B42" s="25" t="s">
+        <v>329</v>
+      </c>
+      <c r="C42" s="9" t="s">
         <v>330</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="D42" s="9" t="s">
         <v>331</v>
-      </c>
-      <c r="D42" s="9" t="s">
-        <v>332</v>
       </c>
       <c r="E42" s="9"/>
       <c r="F42" s="9"/>
@@ -2419,13 +2419,13 @@
         <v>66</v>
       </c>
       <c r="B43" s="25" t="s">
+        <v>332</v>
+      </c>
+      <c r="C43" s="9" t="s">
         <v>333</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="D43" s="9" t="s">
         <v>334</v>
-      </c>
-      <c r="D43" s="9" t="s">
-        <v>335</v>
       </c>
       <c r="E43" s="9"/>
       <c r="F43" s="9"/>
@@ -2435,13 +2435,13 @@
         <v>66</v>
       </c>
       <c r="B44" s="25" t="s">
+        <v>335</v>
+      </c>
+      <c r="C44" s="9" t="s">
         <v>336</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="D44" s="9" t="s">
         <v>337</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>338</v>
       </c>
       <c r="E44" s="9"/>
       <c r="F44" s="9"/>
@@ -2478,7 +2478,7 @@
         <v>102</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="F46" s="9"/>
     </row>
@@ -2630,7 +2630,7 @@
         <v>133</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>134</v>
+        <v>341</v>
       </c>
       <c r="F55" s="9"/>
     </row>
@@ -2639,16 +2639,16 @@
         <v>66</v>
       </c>
       <c r="B56" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="C56" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="D56" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="D56" s="9" t="s">
+      <c r="E56" s="9" t="s">
         <v>137</v>
-      </c>
-      <c r="E56" s="9" t="s">
-        <v>138</v>
       </c>
       <c r="F56" s="9"/>
     </row>
@@ -2657,13 +2657,13 @@
         <v>66</v>
       </c>
       <c r="B57" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="C57" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="D57" s="9" t="s">
         <v>172</v>
-      </c>
-      <c r="D57" s="9" t="s">
-        <v>173</v>
       </c>
       <c r="E57" s="9"/>
       <c r="F57" s="9"/>
@@ -2673,765 +2673,765 @@
         <v>66</v>
       </c>
       <c r="B58" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="C58" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="D58" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="D58" s="9" t="s">
+      <c r="E58" s="9" t="s">
         <v>176</v>
-      </c>
-      <c r="E58" s="9" t="s">
-        <v>177</v>
       </c>
       <c r="F58" s="9"/>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="B59" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="C59" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="D59" s="9" t="s">
         <v>141</v>
-      </c>
-      <c r="D59" s="9" t="s">
-        <v>142</v>
       </c>
       <c r="E59" s="9"/>
       <c r="F59" s="9"/>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B60" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="C60" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="D60" s="9" t="s">
         <v>144</v>
-      </c>
-      <c r="D60" s="9" t="s">
-        <v>145</v>
       </c>
       <c r="E60" s="9"/>
       <c r="F60" s="9"/>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B61" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C61" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="D61" s="9" t="s">
         <v>147</v>
-      </c>
-      <c r="D61" s="9" t="s">
-        <v>148</v>
       </c>
       <c r="E61" s="9"/>
       <c r="F61" s="9"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B62" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C62" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="C62" s="9" t="s">
+      <c r="D62" s="9" t="s">
         <v>150</v>
-      </c>
-      <c r="D62" s="9" t="s">
-        <v>151</v>
       </c>
       <c r="E62" s="9"/>
       <c r="F62" s="9"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B63" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C63" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="C63" s="9" t="s">
+      <c r="D63" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="D63" s="9" t="s">
-        <v>154</v>
       </c>
       <c r="E63" s="9"/>
       <c r="F63" s="9"/>
     </row>
     <row r="64" spans="1:6" ht="70" x14ac:dyDescent="0.2">
       <c r="A64" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B64" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="C64" s="20" t="s">
         <v>155</v>
       </c>
-      <c r="C64" s="20" t="s">
+      <c r="D64" s="20" t="s">
         <v>156</v>
-      </c>
-      <c r="D64" s="20" t="s">
-        <v>157</v>
       </c>
       <c r="E64" s="9"/>
       <c r="F64" s="15" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="70" x14ac:dyDescent="0.2">
       <c r="A65" s="9" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B65" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C65" s="20" t="s">
         <v>159</v>
       </c>
-      <c r="C65" s="20" t="s">
+      <c r="D65" s="20" t="s">
         <v>160</v>
-      </c>
-      <c r="D65" s="20" t="s">
-        <v>161</v>
       </c>
       <c r="E65" s="9"/>
       <c r="F65" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="66" spans="1:6" ht="70" x14ac:dyDescent="0.2">
       <c r="A66" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B66" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B66" s="9" t="s">
+      <c r="C66" s="20" t="s">
         <v>164</v>
       </c>
-      <c r="C66" s="20" t="s">
+      <c r="D66" s="20" t="s">
         <v>165</v>
       </c>
-      <c r="D66" s="20" t="s">
+      <c r="E66" s="15" t="s">
         <v>166</v>
-      </c>
-      <c r="E66" s="15" t="s">
-        <v>167</v>
       </c>
       <c r="F66" s="9"/>
     </row>
     <row r="67" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A67" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B67" s="22" t="s">
+        <v>167</v>
+      </c>
+      <c r="C67" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="C67" s="20" t="s">
+      <c r="D67" s="20" t="s">
         <v>169</v>
-      </c>
-      <c r="D67" s="20" t="s">
-        <v>170</v>
       </c>
       <c r="E67" s="9"/>
       <c r="F67" s="9"/>
     </row>
     <row r="68" spans="1:6" ht="42" x14ac:dyDescent="0.2">
       <c r="A68" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B68" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="C68" s="9" t="s">
         <v>178</v>
       </c>
-      <c r="C68" s="9" t="s">
+      <c r="D68" s="9" t="s">
         <v>179</v>
-      </c>
-      <c r="D68" s="9" t="s">
-        <v>180</v>
       </c>
       <c r="E68" s="9"/>
       <c r="F68" s="15" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="56" x14ac:dyDescent="0.2">
       <c r="A69" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B69" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="C69" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="C69" s="9" t="s">
+      <c r="D69" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="D69" s="9" t="s">
+      <c r="E69" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="E69" s="9" t="s">
+      <c r="F69" s="15" t="s">
         <v>185</v>
-      </c>
-      <c r="F69" s="15" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B70" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="C70" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="D70" s="9" t="s">
         <v>188</v>
-      </c>
-      <c r="D70" s="9" t="s">
-        <v>189</v>
       </c>
       <c r="E70" s="9"/>
       <c r="F70" s="9"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B71" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C71" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="D71" s="9" t="s">
         <v>191</v>
-      </c>
-      <c r="D71" s="9" t="s">
-        <v>192</v>
       </c>
       <c r="E71" s="9"/>
       <c r="F71" s="9"/>
     </row>
     <row r="72" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A72" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B72" s="23" t="s">
+        <v>192</v>
+      </c>
+      <c r="C72" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="D72" s="15" t="s">
         <v>194</v>
-      </c>
-      <c r="D72" s="15" t="s">
-        <v>195</v>
       </c>
       <c r="E72" s="9"/>
       <c r="F72" s="9"/>
     </row>
     <row r="73" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A73" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B73" s="23" t="s">
+        <v>195</v>
+      </c>
+      <c r="C73" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="D73" s="15" t="s">
         <v>197</v>
-      </c>
-      <c r="D73" s="15" t="s">
-        <v>198</v>
       </c>
       <c r="E73" s="9"/>
       <c r="F73" s="9"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="B74" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="B74" s="9" t="s">
+      <c r="C74" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="D74" s="9" t="s">
         <v>201</v>
-      </c>
-      <c r="D74" s="9" t="s">
-        <v>202</v>
       </c>
       <c r="E74" s="9"/>
       <c r="F74" s="9"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B75" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="C75" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="C75" s="9" t="s">
+      <c r="D75" s="9" t="s">
         <v>204</v>
-      </c>
-      <c r="D75" s="9" t="s">
-        <v>205</v>
       </c>
       <c r="E75" s="9"/>
       <c r="F75" s="9"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B76" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="C76" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="C76" s="9" t="s">
+      <c r="D76" s="9" t="s">
         <v>207</v>
-      </c>
-      <c r="D76" s="9" t="s">
-        <v>208</v>
       </c>
       <c r="E76" s="9"/>
       <c r="F76" s="9"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B77" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="C77" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="C77" s="9" t="s">
+      <c r="D77" s="9" t="s">
         <v>210</v>
-      </c>
-      <c r="D77" s="9" t="s">
-        <v>211</v>
       </c>
       <c r="E77" s="9"/>
       <c r="F77" s="9"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B78" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="C78" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="D78" s="9" t="s">
         <v>212</v>
-      </c>
-      <c r="C78" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="D78" s="9" t="s">
-        <v>213</v>
       </c>
       <c r="E78" s="9"/>
       <c r="F78" s="9"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="9" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B79" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="C79" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="C79" s="9" t="s">
+      <c r="D79" s="9" t="s">
         <v>215</v>
-      </c>
-      <c r="D79" s="9" t="s">
-        <v>216</v>
       </c>
       <c r="E79" s="9"/>
       <c r="F79" s="9"/>
     </row>
     <row r="80" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A80" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="B80" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="B80" s="9" t="s">
+      <c r="C80" s="9" t="s">
         <v>218</v>
       </c>
-      <c r="C80" s="9" t="s">
+      <c r="D80" s="15" t="s">
         <v>219</v>
       </c>
-      <c r="D80" s="15" t="s">
+      <c r="E80" s="9" t="s">
         <v>220</v>
-      </c>
-      <c r="E80" s="9" t="s">
-        <v>221</v>
       </c>
       <c r="F80" s="9"/>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B81" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="C81" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="C81" s="9" t="s">
+      <c r="D81" s="9" t="s">
         <v>223</v>
-      </c>
-      <c r="D81" s="9" t="s">
-        <v>224</v>
       </c>
       <c r="E81" s="9"/>
       <c r="F81" s="9"/>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B82" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="C82" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="C82" s="9" t="s">
+      <c r="D82" s="9" t="s">
         <v>226</v>
-      </c>
-      <c r="D82" s="9" t="s">
-        <v>227</v>
       </c>
       <c r="E82" s="9"/>
       <c r="F82" s="9"/>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B83" s="9" t="s">
+        <v>227</v>
+      </c>
+      <c r="C83" s="9" t="s">
         <v>228</v>
       </c>
-      <c r="C83" s="9" t="s">
+      <c r="D83" s="9" t="s">
         <v>229</v>
-      </c>
-      <c r="D83" s="9" t="s">
-        <v>230</v>
       </c>
       <c r="E83" s="9"/>
       <c r="F83" s="9"/>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B84" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="C84" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="C84" s="9" t="s">
+      <c r="D84" s="9" t="s">
         <v>232</v>
-      </c>
-      <c r="D84" s="9" t="s">
-        <v>233</v>
       </c>
       <c r="E84" s="9"/>
       <c r="F84" s="9"/>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B85" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="C85" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="C85" s="9" t="s">
+      <c r="D85" s="9" t="s">
         <v>235</v>
-      </c>
-      <c r="D85" s="9" t="s">
-        <v>236</v>
       </c>
       <c r="E85" s="9"/>
       <c r="F85" s="9"/>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="9" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B86" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="C86" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="C86" s="9" t="s">
+      <c r="D86" s="9" t="s">
         <v>238</v>
-      </c>
-      <c r="D86" s="9" t="s">
-        <v>239</v>
       </c>
       <c r="E86" s="9"/>
       <c r="F86" s="9"/>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="B87" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="B87" s="9" t="s">
+      <c r="C87" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="C87" s="9" t="s">
+      <c r="D87" s="9" t="s">
         <v>242</v>
-      </c>
-      <c r="D87" s="9" t="s">
-        <v>243</v>
       </c>
       <c r="E87" s="9"/>
       <c r="F87" s="9"/>
     </row>
     <row r="88" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A88" s="15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B88" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="C88" s="15" t="s">
         <v>244</v>
       </c>
-      <c r="C88" s="15" t="s">
+      <c r="D88" s="15" t="s">
         <v>245</v>
       </c>
-      <c r="D88" s="15" t="s">
+      <c r="E88" s="9" t="s">
         <v>246</v>
-      </c>
-      <c r="E88" s="9" t="s">
-        <v>247</v>
       </c>
       <c r="F88" s="9"/>
     </row>
     <row r="89" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A89" s="15" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B89" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="C89" s="15" t="s">
         <v>248</v>
       </c>
-      <c r="C89" s="15" t="s">
+      <c r="D89" s="15" t="s">
         <v>249</v>
       </c>
-      <c r="D89" s="15" t="s">
+      <c r="E89" s="15" t="s">
         <v>250</v>
-      </c>
-      <c r="E89" s="15" t="s">
-        <v>251</v>
       </c>
       <c r="F89" s="9"/>
     </row>
     <row r="90" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A90" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="B90" s="22" t="s">
         <v>252</v>
       </c>
-      <c r="B90" s="22" t="s">
+      <c r="C90" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="C90" s="15" t="s">
+      <c r="D90" s="15" t="s">
         <v>254</v>
-      </c>
-      <c r="D90" s="15" t="s">
-        <v>255</v>
       </c>
       <c r="E90" s="9"/>
       <c r="F90" s="9"/>
     </row>
     <row r="91" spans="1:6" ht="42" x14ac:dyDescent="0.2">
       <c r="A91" s="15" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B91" s="22" t="s">
+        <v>255</v>
+      </c>
+      <c r="C91" s="15" t="s">
         <v>256</v>
       </c>
-      <c r="C91" s="15" t="s">
+      <c r="D91" s="15" t="s">
         <v>257</v>
       </c>
-      <c r="D91" s="15" t="s">
+      <c r="E91" s="9" t="s">
         <v>258</v>
-      </c>
-      <c r="E91" s="9" t="s">
-        <v>259</v>
       </c>
       <c r="F91" s="9"/>
     </row>
     <row r="92" spans="1:6" ht="112" x14ac:dyDescent="0.2">
       <c r="A92" s="9" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B92" s="23" t="s">
+        <v>259</v>
+      </c>
+      <c r="C92" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="C92" s="9" t="s">
+      <c r="D92" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="D92" s="9" t="s">
+      <c r="E92" s="15" t="s">
         <v>262</v>
-      </c>
-      <c r="E92" s="15" t="s">
-        <v>263</v>
       </c>
       <c r="F92" s="9"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="B93" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="B93" s="9" t="s">
+      <c r="C93" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="C93" s="9" t="s">
+      <c r="D93" s="15" t="s">
         <v>266</v>
-      </c>
-      <c r="D93" s="15" t="s">
-        <v>267</v>
       </c>
       <c r="E93" s="9"/>
       <c r="F93" s="9"/>
     </row>
     <row r="94" spans="1:6" ht="42" x14ac:dyDescent="0.2">
       <c r="A94" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B94" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="C94" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="D94" s="15" t="s">
         <v>268</v>
       </c>
-      <c r="C94" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="D94" s="15" t="s">
+      <c r="E94" s="9" t="s">
         <v>269</v>
-      </c>
-      <c r="E94" s="9" t="s">
-        <v>270</v>
       </c>
       <c r="F94" s="9"/>
     </row>
     <row r="95" spans="1:6" ht="84" x14ac:dyDescent="0.2">
       <c r="A95" s="9" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B95" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="C95" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="C95" s="9" t="s">
+      <c r="D95" s="15" t="s">
         <v>272</v>
       </c>
-      <c r="D95" s="15" t="s">
+      <c r="E95" s="15" t="s">
         <v>273</v>
-      </c>
-      <c r="E95" s="15" t="s">
-        <v>274</v>
       </c>
       <c r="F95" s="9"/>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="B96" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B96" s="9" t="s">
+      <c r="C96" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="C96" s="9" t="s">
+      <c r="D96" s="9" t="s">
         <v>277</v>
-      </c>
-      <c r="D96" s="9" t="s">
-        <v>278</v>
       </c>
       <c r="E96" s="15"/>
       <c r="F96" s="9"/>
     </row>
     <row r="97" spans="1:6" ht="42" x14ac:dyDescent="0.2">
       <c r="A97" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B97" s="24" t="s">
+        <v>278</v>
+      </c>
+      <c r="C97" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="C97" s="9" t="s">
+      <c r="D97" s="15" t="s">
         <v>280</v>
       </c>
-      <c r="D97" s="15" t="s">
+      <c r="E97" s="15" t="s">
         <v>281</v>
-      </c>
-      <c r="E97" s="15" t="s">
-        <v>282</v>
       </c>
       <c r="F97" s="9"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" s="9" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B98" s="24" t="s">
+        <v>282</v>
+      </c>
+      <c r="C98" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="C98" s="9" t="s">
+      <c r="D98" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="D98" s="9" t="s">
-        <v>285</v>
       </c>
       <c r="E98" s="9"/>
       <c r="F98" s="9"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="B99" s="9" t="s">
         <v>286</v>
       </c>
-      <c r="B99" s="9" t="s">
+      <c r="C99" s="9" t="s">
         <v>287</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="D99" s="9" t="s">
         <v>288</v>
-      </c>
-      <c r="D99" s="9" t="s">
-        <v>289</v>
       </c>
       <c r="E99" s="9"/>
       <c r="F99" s="9"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B100" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="C100" s="9" t="s">
         <v>290</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="D100" s="9" t="s">
         <v>291</v>
       </c>
-      <c r="D100" s="9" t="s">
+      <c r="E100" s="9" t="s">
         <v>292</v>
-      </c>
-      <c r="E100" s="9" t="s">
-        <v>293</v>
       </c>
       <c r="F100" s="9"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B101" s="9" t="s">
+        <v>293</v>
+      </c>
+      <c r="C101" s="9" t="s">
         <v>294</v>
       </c>
-      <c r="C101" s="9" t="s">
+      <c r="D101" s="9" t="s">
         <v>295</v>
-      </c>
-      <c r="D101" s="9" t="s">
-        <v>296</v>
       </c>
       <c r="E101" s="9"/>
       <c r="F101" s="9"/>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B102" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="C102" s="9" t="s">
         <v>297</v>
       </c>
-      <c r="C102" s="9" t="s">
+      <c r="D102" s="9" t="s">
         <v>298</v>
-      </c>
-      <c r="D102" s="9" t="s">
-        <v>299</v>
       </c>
       <c r="E102" s="9"/>
       <c r="F102" s="9"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B103" s="9" t="s">
+        <v>299</v>
+      </c>
+      <c r="C103" s="9" t="s">
         <v>300</v>
       </c>
-      <c r="C103" s="9" t="s">
+      <c r="D103" s="9" t="s">
         <v>301</v>
-      </c>
-      <c r="D103" s="9" t="s">
-        <v>302</v>
       </c>
       <c r="E103" s="9"/>
       <c r="F103" s="9"/>

</xml_diff>